<commit_message>
Add live precious-metal spot prices (gold, silver)
</commit_message>
<xml_diff>
--- a/sample_tracker.xlsx
+++ b/sample_tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79d77e64bffb398c/Documents/Python files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79d77e64bffb398c/Documents/Python/Python files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_F00F239ABF17E63606E8A8B3F15EF2318793852F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FBB9574-776D-489C-8FAE-255CE5EB0CDD}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_F00F239ABF17E63606E8A8B3F15EF2318793852F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81B104A8-C3EA-4095-9C31-3CF1B6DC8257}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>item</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Gold miners ETF</t>
   </si>
   <si>
-    <t>Precious metals</t>
-  </si>
-  <si>
     <t>cash</t>
   </si>
   <si>
@@ -68,6 +65,18 @@
   </si>
   <si>
     <t>GDX</t>
+  </si>
+  <si>
+    <t>Silver (oz)</t>
+  </si>
+  <si>
+    <t>Gold (oz)</t>
+  </si>
+  <si>
+    <t>SI=F</t>
+  </si>
+  <si>
+    <t>GC=F</t>
   </si>
 </sst>
 </file>
@@ -409,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" bestFit="1" customWidth="1"/>
@@ -440,7 +449,7 @@
         <v>5000</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -451,7 +460,7 @@
         <v>5000</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -462,10 +471,10 @@
         <v>5000</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>50</v>
@@ -479,10 +488,10 @@
         <v>5000</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>50</v>
@@ -490,13 +499,36 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B6">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7">
+        <v>4000</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>